<commit_message>
update: monthly data 週三 2026/10/07
</commit_message>
<xml_diff>
--- a/data/AIRSPACE_線下通路_行銷排程_含甘特圖_2025-2026.xlsx
+++ b/data/AIRSPACE_線下通路_行銷排程_含甘特圖_2025-2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="486">
   <si>
     <t>年度</t>
   </si>
@@ -1384,10 +1384,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>08/17-09/13</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>08/17-08/30 春夏鞋款全館單件65折 (排除聯名款) 大碼商品全館單件85折</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1405,6 +1401,93 @@
   </si>
   <si>
     <t>7/9-7/26 部分店櫃適用 一般會員/過路客滿3200贈玩總行李吊牌 VIP/SVIP滿2500贈玩總行李吊牌 左營新光店、台中漢神店、嘉義秀泰店、新台南FOCUS店</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>09月</t>
+  </si>
+  <si>
+    <t>09/07-09/13</t>
+  </si>
+  <si>
+    <t>09/07-09/13 門網同步 (包含IP店櫃) 全館三件85折</t>
+  </si>
+  <si>
+    <t>甜甜價/體驗價/組合價(包含買單件)*不列入三件折扣</t>
+  </si>
+  <si>
+    <t>2026/08/31郵件</t>
+  </si>
+  <si>
+    <t>體驗價*不列入單件折扣</t>
+  </si>
+  <si>
+    <t>09/17-09/28</t>
+  </si>
+  <si>
+    <t>周慶店櫃活動 (不與其他活動併用) 周慶活動 適用店櫃 滿2500折300 (88折) 滿3800折600 (84折) 滿5000折850 (83折) 09/17-09/28 台中遠百 09/24-10/04 夢時代體系 09/24-10/04 統領體系 09/24-10/04 台茂體系</t>
+  </si>
+  <si>
+    <t>首四日*滿2000送湯姆貓手機鍊 (非IP店);整檔期*滿2000送崔弟造型筆 (IP店)</t>
+  </si>
+  <si>
+    <t>09/07-09/30</t>
+  </si>
+  <si>
+    <t>2026/09/07郵件</t>
+  </si>
+  <si>
+    <t>09/07-09/28</t>
+  </si>
+  <si>
+    <t>09/14-09/23</t>
+  </si>
+  <si>
+    <t>09/14-09/23 門網同步 (包含IP店櫃) 全館小物兩件85折 (聯名配件)</t>
+  </si>
+  <si>
+    <t>外採IP小物/寄賣商品/服裝配件 *不列入折扣 (活動貨組如附件)</t>
+  </si>
+  <si>
+    <t>2026/09/14郵件</t>
+  </si>
+  <si>
+    <t>25月</t>
+  </si>
+  <si>
+    <t>2025/08/01起 官網下單門市取貨獨家 凡於官網下單門市取貨者 當日到店取貨且在門市不限消費金額現折100 POS操作：輸入會員條碼→再輸入折扣碼【PICKUP100】</t>
+  </si>
+  <si>
+    <t>2026/09/24郵件</t>
+  </si>
+  <si>
+    <t>09/29-11/01</t>
+  </si>
+  <si>
+    <t>一單可複數件加購 (同時可加購不同款式、也可同一款式加購兩個以上)</t>
+  </si>
+  <si>
+    <t>09/07-09/30 門市獨家加碼活動 精選春夏鞋款單雙現折500</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>凡購買任一商品享舒芙蕾內衣加購價$399</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>08/17-09/06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>09/07-09/28 門網同步活動時間調整 (包含IP店櫃) 全館泳裝單件85折</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>09/24-09/28</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>09/24-09/28全館單件88折 (門網同步) 滿2500再折150 (門市獨加加碼)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1414,9 +1497,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="176" formatCode="m/d"/>
-    <numFmt numFmtId="181" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
+    <numFmt numFmtId="177" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1441,6 +1524,13 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
       <charset val="136"/>
@@ -1529,7 +1619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1576,14 +1666,137 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="181" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="45">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDEEBF7"/>
+          <bgColor rgb="FFDEEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBDD7EE"/>
+          <bgColor rgb="FFBDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDEEBF7"/>
+          <bgColor rgb="FFDEEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2036,7 +2249,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I982"/>
+  <dimension ref="A1:I971"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="6" style="4" customWidth="1"/>
@@ -6499,7 +6712,7 @@
         <v>397</v>
       </c>
       <c r="E154" s="15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F154" s="15" t="s">
         <v>12</v>
@@ -6528,7 +6741,7 @@
         <v>95</v>
       </c>
       <c r="E155" s="15" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F155" s="15" t="s">
         <v>12</v>
@@ -6557,7 +6770,7 @@
         <v>95</v>
       </c>
       <c r="E156" s="15" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F156" s="15" t="s">
         <v>436</v>
@@ -6679,7 +6892,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="4">
         <v>2026</v>
       </c>
@@ -6693,7 +6906,7 @@
         <v>22</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F161" s="4" t="s">
         <v>12</v>
@@ -6705,7 +6918,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="4">
         <v>2026</v>
       </c>
@@ -6713,7 +6926,7 @@
         <v>135</v>
       </c>
       <c r="C162" s="16" t="s">
-        <v>454</v>
+        <v>482</v>
       </c>
       <c r="D162" s="4" t="s">
         <v>439</v>
@@ -6731,7 +6944,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="4">
         <v>2026</v>
       </c>
@@ -6745,7 +6958,7 @@
         <v>22</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F163" s="4" t="s">
         <v>12</v>
@@ -6757,7 +6970,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="4">
         <v>2026</v>
       </c>
@@ -6783,18 +6996,267 @@
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B165" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C165" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="D165" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E165" s="17" t="s">
+        <v>461</v>
+      </c>
+      <c r="F165" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G165" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H165" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="I165" s="17" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B166" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C166" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="D166" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E166" s="17" t="s">
+        <v>480</v>
+      </c>
+      <c r="F166" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="G166" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="H166" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="I166" s="17" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B167" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C167" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="D167" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E167" s="17" t="s">
+        <v>483</v>
+      </c>
+      <c r="F167" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G167" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="H167" s="17" t="s">
+        <v>464</v>
+      </c>
+      <c r="I167" s="17" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B168" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C168" s="17" t="s">
+        <v>484</v>
+      </c>
+      <c r="D168" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="E168" s="17" t="s">
+        <v>485</v>
+      </c>
+      <c r="F168" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G168" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H168" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="I168" s="17" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B169" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C169" s="17" t="s">
+        <v>465</v>
+      </c>
+      <c r="D169" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E169" s="17" t="s">
+        <v>466</v>
+      </c>
+      <c r="F169" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G169" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H169" s="17" t="s">
+        <v>467</v>
+      </c>
+      <c r="I169" s="17" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B170" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C170" s="16" t="s">
+        <v>482</v>
+      </c>
+      <c r="D170" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="E170" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="F170" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G170" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H170" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B171" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C171" s="17" t="s">
+        <v>471</v>
+      </c>
+      <c r="D171" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E171" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="F171" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G171" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H171" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="I171" s="17" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B172" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="C172" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D172" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="E172" s="17" t="s">
+        <v>476</v>
+      </c>
+      <c r="F172" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G172" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H172" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="I172" s="17" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="17">
+        <v>2026</v>
+      </c>
+      <c r="B173" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="C173" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="D173" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="E173" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="F173" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G173" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="H173" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="I173" s="17" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7590,17 +8052,6 @@
     <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:I151">
     <sortState ref="A2:I164">
@@ -7608,77 +8059,152 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="29" priority="16" stopIfTrue="1" operator="equal">
+      <formula>"調整後"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="28" priority="17" stopIfTrue="1" operator="equal">
+      <formula>"再次調整"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="27" priority="18" stopIfTrue="1" operator="equal">
+      <formula>"延長"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="26" priority="19" stopIfTrue="1" operator="equal">
+      <formula>"再次延長"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="25" priority="20" stopIfTrue="1" operator="equal">
+      <formula>"加碼"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="24" priority="21" stopIfTrue="1" operator="equal">
+      <formula>"獨家加碼"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="23" priority="22" stopIfTrue="1" operator="equal">
+      <formula>"搶先開跑"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="22" priority="23" stopIfTrue="1" operator="equal">
+      <formula>"取消"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="21" priority="24" stopIfTrue="1" operator="equal">
+      <formula>"補充"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="20" priority="25" stopIfTrue="1" operator="equal">
+      <formula>"長期"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="19" priority="26" stopIfTrue="1" operator="equal">
+      <formula>"日期調整"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="18" priority="27" stopIfTrue="1" operator="equal">
+      <formula>"系統調整"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="17" priority="28" stopIfTrue="1" operator="equal">
+      <formula>"原訂(後改)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="16" priority="29" stopIfTrue="1" operator="equal">
+      <formula>"原訂(後延長)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G171:G971 G2:G169">
+    <cfRule type="cellIs" dxfId="15" priority="30" stopIfTrue="1" operator="equal">
+      <formula>"原訂(後取消)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="14" priority="1" stopIfTrue="1" operator="equal">
       <formula>"調整後"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="13" priority="2" stopIfTrue="1" operator="equal">
       <formula>"再次調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="12" priority="3" stopIfTrue="1" operator="equal">
       <formula>"延長"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="11" priority="4" stopIfTrue="1" operator="equal">
       <formula>"再次延長"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="10" priority="5" stopIfTrue="1" operator="equal">
       <formula>"加碼"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="9" priority="6" stopIfTrue="1" operator="equal">
       <formula>"獨家加碼"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="8" priority="7" stopIfTrue="1" operator="equal">
       <formula>"搶先開跑"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="7" priority="8" stopIfTrue="1" operator="equal">
       <formula>"取消"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="6" priority="9" stopIfTrue="1" operator="equal">
       <formula>"補充"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="5" priority="10" stopIfTrue="1" operator="equal">
       <formula>"長期"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="4" priority="11" stopIfTrue="1" operator="equal">
       <formula>"日期調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="3" priority="12" stopIfTrue="1" operator="equal">
       <formula>"系統調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="2" priority="13" stopIfTrue="1" operator="equal">
       <formula>"原訂(後改)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="1" priority="14" stopIfTrue="1" operator="equal">
       <formula>"原訂(後延長)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G982">
+  <conditionalFormatting sqref="G170">
     <cfRule type="cellIs" dxfId="0" priority="15" stopIfTrue="1" operator="equal">
       <formula>"原訂(後取消)"</formula>
     </cfRule>

</xml_diff>